<commit_message>
Jesus is the way
</commit_message>
<xml_diff>
--- a/vignettes/best_models.xlsx
+++ b/vignettes/best_models.xlsx
@@ -351,7 +351,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:N52"/>
+  <dimension ref="A1:AB52"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -417,12 +417,82 @@
       </c>
       <c r="M1" s="1" t="inlineStr">
         <is>
+          <t>n_success_folds</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>n_failed_folds</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>n_predictions</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
           <t>n_success</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>n_failed</t>
+        </is>
+      </c>
+      <c r="R1" s="1" t="inlineStr">
+        <is>
+          <t>n_warning_folds</t>
+        </is>
+      </c>
+      <c r="S1" s="1" t="inlineStr">
+        <is>
+          <t>warning_rate</t>
+        </is>
+      </c>
+      <c r="T1" s="1" t="inlineStr">
+        <is>
+          <t>n_warning_events</t>
+        </is>
+      </c>
+      <c r="U1" s="1" t="inlineStr">
+        <is>
+          <t>n_knot_warning_folds</t>
+        </is>
+      </c>
+      <c r="V1" s="1" t="inlineStr">
+        <is>
+          <t>n_convergence_warning_folds</t>
+        </is>
+      </c>
+      <c r="W1" s="1" t="inlineStr">
+        <is>
+          <t>n_hessian_warning_folds</t>
+        </is>
+      </c>
+      <c r="X1" s="1" t="inlineStr">
+        <is>
+          <t>n_other_warning_folds</t>
+        </is>
+      </c>
+      <c r="Y1" s="1" t="inlineStr">
+        <is>
+          <t>n_knot_warning_events</t>
+        </is>
+      </c>
+      <c r="Z1" s="1" t="inlineStr">
+        <is>
+          <t>n_convergence_warning_events</t>
+        </is>
+      </c>
+      <c r="AA1" s="1" t="inlineStr">
+        <is>
+          <t>n_hessian_warning_events</t>
+        </is>
+      </c>
+      <c r="AB1" s="1" t="inlineStr">
+        <is>
+          <t>n_other_warning_events</t>
         </is>
       </c>
     </row>
@@ -448,19 +518,19 @@
         <v>3</v>
       </c>
       <c r="G2">
-        <v>0.9799852872109197</v>
+        <v>0.979950158164056</v>
       </c>
       <c r="H2">
-        <v>0.9997286328642065</v>
+        <v>0.9997242448267788</v>
       </c>
       <c r="I2">
-        <v>0.9802512951972552</v>
+        <v>0.9802204590265299</v>
       </c>
       <c r="J2">
-        <v>0.05287834631584271</v>
+        <v>0.05291964298881337</v>
       </c>
       <c r="K2">
-        <v>0.03814998576608081</v>
+        <v>0.03821928249386558</v>
       </c>
       <c r="L2">
         <v>520</v>
@@ -469,6 +539,48 @@
         <v>520</v>
       </c>
       <c r="N2">
+        <v>0</v>
+      </c>
+      <c r="O2">
+        <v>520</v>
+      </c>
+      <c r="P2">
+        <v>520</v>
+      </c>
+      <c r="Q2">
+        <v>0</v>
+      </c>
+      <c r="R2">
+        <v>520</v>
+      </c>
+      <c r="S2">
+        <v>1</v>
+      </c>
+      <c r="T2">
+        <v>1010</v>
+      </c>
+      <c r="U2">
+        <v>520</v>
+      </c>
+      <c r="V2">
+        <v>490</v>
+      </c>
+      <c r="W2">
+        <v>0</v>
+      </c>
+      <c r="X2">
+        <v>0</v>
+      </c>
+      <c r="Y2">
+        <v>520</v>
+      </c>
+      <c r="Z2">
+        <v>490</v>
+      </c>
+      <c r="AA2">
+        <v>0</v>
+      </c>
+      <c r="AB2">
         <v>0</v>
       </c>
     </row>
@@ -494,19 +606,19 @@
         <v>3</v>
       </c>
       <c r="G3">
-        <v>0.9782914641588488</v>
+        <v>0.9782916129408498</v>
       </c>
       <c r="H3">
-        <v>0.9996410864462579</v>
+        <v>0.9996410900831298</v>
       </c>
       <c r="I3">
-        <v>0.9786427122925615</v>
+        <v>0.9786428575675048</v>
       </c>
       <c r="J3">
-        <v>0.05497642521963983</v>
+        <v>0.05497623947223665</v>
       </c>
       <c r="K3">
-        <v>0.03951970289620614</v>
+        <v>0.03951957186975079</v>
       </c>
       <c r="L3">
         <v>520</v>
@@ -515,6 +627,48 @@
         <v>520</v>
       </c>
       <c r="N3">
+        <v>0</v>
+      </c>
+      <c r="O3">
+        <v>520</v>
+      </c>
+      <c r="P3">
+        <v>520</v>
+      </c>
+      <c r="Q3">
+        <v>0</v>
+      </c>
+      <c r="R3">
+        <v>520</v>
+      </c>
+      <c r="S3">
+        <v>1</v>
+      </c>
+      <c r="T3">
+        <v>523</v>
+      </c>
+      <c r="U3">
+        <v>520</v>
+      </c>
+      <c r="V3">
+        <v>3</v>
+      </c>
+      <c r="W3">
+        <v>0</v>
+      </c>
+      <c r="X3">
+        <v>0</v>
+      </c>
+      <c r="Y3">
+        <v>520</v>
+      </c>
+      <c r="Z3">
+        <v>3</v>
+      </c>
+      <c r="AA3">
+        <v>0</v>
+      </c>
+      <c r="AB3">
         <v>0</v>
       </c>
     </row>
@@ -540,19 +694,19 @@
         <v>3</v>
       </c>
       <c r="G4">
-        <v>0.9701844239157018</v>
+        <v>0.9701868525892332</v>
       </c>
       <c r="H4">
-        <v>0.9993803604311973</v>
+        <v>0.9993807576911117</v>
       </c>
       <c r="I4">
-        <v>0.9707859613101678</v>
+        <v>0.9707880055952591</v>
       </c>
       <c r="J4">
-        <v>0.06417070152586207</v>
+        <v>0.06416849493374555</v>
       </c>
       <c r="K4">
-        <v>0.04748697035921893</v>
+        <v>0.04748532025333416</v>
       </c>
       <c r="L4">
         <v>520</v>
@@ -561,6 +715,48 @@
         <v>520</v>
       </c>
       <c r="N4">
+        <v>0</v>
+      </c>
+      <c r="O4">
+        <v>520</v>
+      </c>
+      <c r="P4">
+        <v>520</v>
+      </c>
+      <c r="Q4">
+        <v>0</v>
+      </c>
+      <c r="R4">
+        <v>520</v>
+      </c>
+      <c r="S4">
+        <v>1</v>
+      </c>
+      <c r="T4">
+        <v>530</v>
+      </c>
+      <c r="U4">
+        <v>520</v>
+      </c>
+      <c r="V4">
+        <v>10</v>
+      </c>
+      <c r="W4">
+        <v>0</v>
+      </c>
+      <c r="X4">
+        <v>0</v>
+      </c>
+      <c r="Y4">
+        <v>520</v>
+      </c>
+      <c r="Z4">
+        <v>10</v>
+      </c>
+      <c r="AA4">
+        <v>0</v>
+      </c>
+      <c r="AB4">
         <v>0</v>
       </c>
     </row>
@@ -586,19 +782,19 @@
         <v>3</v>
       </c>
       <c r="G5">
-        <v>0.9687742254063078</v>
+        <v>0.9687742178427846</v>
       </c>
       <c r="H5">
-        <v>0.999263977391457</v>
+        <v>0.99926394184089</v>
       </c>
       <c r="I5">
-        <v>0.9694877903387035</v>
+        <v>0.9694878172608372</v>
       </c>
       <c r="J5">
-        <v>0.06557174317758258</v>
+        <v>0.06557171504657712</v>
       </c>
       <c r="K5">
-        <v>0.04834567387115964</v>
+        <v>0.04834563651066225</v>
       </c>
       <c r="L5">
         <v>520</v>
@@ -607,6 +803,48 @@
         <v>520</v>
       </c>
       <c r="N5">
+        <v>0</v>
+      </c>
+      <c r="O5">
+        <v>520</v>
+      </c>
+      <c r="P5">
+        <v>520</v>
+      </c>
+      <c r="Q5">
+        <v>0</v>
+      </c>
+      <c r="R5">
+        <v>520</v>
+      </c>
+      <c r="S5">
+        <v>1</v>
+      </c>
+      <c r="T5">
+        <v>520</v>
+      </c>
+      <c r="U5">
+        <v>520</v>
+      </c>
+      <c r="V5">
+        <v>0</v>
+      </c>
+      <c r="W5">
+        <v>0</v>
+      </c>
+      <c r="X5">
+        <v>0</v>
+      </c>
+      <c r="Y5">
+        <v>520</v>
+      </c>
+      <c r="Z5">
+        <v>0</v>
+      </c>
+      <c r="AA5">
+        <v>0</v>
+      </c>
+      <c r="AB5">
         <v>0</v>
       </c>
     </row>
@@ -632,19 +870,19 @@
         <v>3</v>
       </c>
       <c r="G6">
-        <v>0.9522659401348015</v>
+        <v>0.952265797576562</v>
       </c>
       <c r="H6">
-        <v>0.998231705086328</v>
+        <v>0.9982316178154013</v>
       </c>
       <c r="I6">
-        <v>0.9539528100366724</v>
+        <v>0.9539527506257176</v>
       </c>
       <c r="J6">
-        <v>0.08027338327304794</v>
+        <v>0.08027343312751634</v>
       </c>
       <c r="K6">
-        <v>0.05770640487944699</v>
+        <v>0.05770645164938885</v>
       </c>
       <c r="L6">
         <v>520</v>
@@ -653,6 +891,48 @@
         <v>520</v>
       </c>
       <c r="N6">
+        <v>0</v>
+      </c>
+      <c r="O6">
+        <v>520</v>
+      </c>
+      <c r="P6">
+        <v>520</v>
+      </c>
+      <c r="Q6">
+        <v>0</v>
+      </c>
+      <c r="R6">
+        <v>520</v>
+      </c>
+      <c r="S6">
+        <v>1</v>
+      </c>
+      <c r="T6">
+        <v>520</v>
+      </c>
+      <c r="U6">
+        <v>520</v>
+      </c>
+      <c r="V6">
+        <v>0</v>
+      </c>
+      <c r="W6">
+        <v>0</v>
+      </c>
+      <c r="X6">
+        <v>0</v>
+      </c>
+      <c r="Y6">
+        <v>520</v>
+      </c>
+      <c r="Z6">
+        <v>0</v>
+      </c>
+      <c r="AA6">
+        <v>0</v>
+      </c>
+      <c r="AB6">
         <v>0</v>
       </c>
     </row>
@@ -678,19 +958,19 @@
         <v>3</v>
       </c>
       <c r="G7">
-        <v>0.9492879984236559</v>
+        <v>0.9492879323778345</v>
       </c>
       <c r="H7">
-        <v>0.9978859331066586</v>
+        <v>0.9978858149749</v>
       </c>
       <c r="I7">
-        <v>0.9512991083743352</v>
+        <v>0.9512991548053141</v>
       </c>
       <c r="J7">
-        <v>0.08253419146750307</v>
+        <v>0.08253415430104309</v>
       </c>
       <c r="K7">
-        <v>0.05886412732857104</v>
+        <v>0.05886408240683829</v>
       </c>
       <c r="L7">
         <v>520</v>
@@ -699,6 +979,48 @@
         <v>520</v>
       </c>
       <c r="N7">
+        <v>0</v>
+      </c>
+      <c r="O7">
+        <v>520</v>
+      </c>
+      <c r="P7">
+        <v>520</v>
+      </c>
+      <c r="Q7">
+        <v>0</v>
+      </c>
+      <c r="R7">
+        <v>520</v>
+      </c>
+      <c r="S7">
+        <v>1</v>
+      </c>
+      <c r="T7">
+        <v>520</v>
+      </c>
+      <c r="U7">
+        <v>520</v>
+      </c>
+      <c r="V7">
+        <v>0</v>
+      </c>
+      <c r="W7">
+        <v>0</v>
+      </c>
+      <c r="X7">
+        <v>0</v>
+      </c>
+      <c r="Y7">
+        <v>520</v>
+      </c>
+      <c r="Z7">
+        <v>0</v>
+      </c>
+      <c r="AA7">
+        <v>0</v>
+      </c>
+      <c r="AB7">
         <v>0</v>
       </c>
     </row>
@@ -724,13 +1046,13 @@
         <v>2</v>
       </c>
       <c r="G8">
-        <v>0.8590465982602428</v>
+        <v>0.8590462606372582</v>
       </c>
       <c r="H8">
-        <v>0.9863059844669356</v>
+        <v>0.9863055968283946</v>
       </c>
       <c r="I8">
-        <v>0.8709737259928803</v>
+        <v>0.8709737259928801</v>
       </c>
       <c r="J8">
         <v>0.1315838789232578</v>
@@ -745,6 +1067,48 @@
         <v>520</v>
       </c>
       <c r="N8">
+        <v>0</v>
+      </c>
+      <c r="O8">
+        <v>520</v>
+      </c>
+      <c r="P8">
+        <v>520</v>
+      </c>
+      <c r="Q8">
+        <v>0</v>
+      </c>
+      <c r="R8">
+        <v>0</v>
+      </c>
+      <c r="S8">
+        <v>0</v>
+      </c>
+      <c r="T8">
+        <v>0</v>
+      </c>
+      <c r="U8">
+        <v>0</v>
+      </c>
+      <c r="V8">
+        <v>0</v>
+      </c>
+      <c r="W8">
+        <v>0</v>
+      </c>
+      <c r="X8">
+        <v>0</v>
+      </c>
+      <c r="Y8">
+        <v>0</v>
+      </c>
+      <c r="Z8">
+        <v>0</v>
+      </c>
+      <c r="AA8">
+        <v>0</v>
+      </c>
+      <c r="AB8">
         <v>0</v>
       </c>
     </row>
@@ -770,13 +1134,13 @@
         <v>2</v>
       </c>
       <c r="G9">
-        <v>0.8575087732687594</v>
+        <v>0.857508440646641</v>
       </c>
       <c r="H9">
-        <v>0.9868661663457738</v>
+        <v>0.9868657835467578</v>
       </c>
       <c r="I9">
-        <v>0.8689210376357246</v>
+        <v>0.8689210376357245</v>
       </c>
       <c r="J9">
         <v>0.1324930450251554</v>
@@ -791,6 +1155,48 @@
         <v>520</v>
       </c>
       <c r="N9">
+        <v>0</v>
+      </c>
+      <c r="O9">
+        <v>520</v>
+      </c>
+      <c r="P9">
+        <v>520</v>
+      </c>
+      <c r="Q9">
+        <v>0</v>
+      </c>
+      <c r="R9">
+        <v>0</v>
+      </c>
+      <c r="S9">
+        <v>0</v>
+      </c>
+      <c r="T9">
+        <v>0</v>
+      </c>
+      <c r="U9">
+        <v>0</v>
+      </c>
+      <c r="V9">
+        <v>0</v>
+      </c>
+      <c r="W9">
+        <v>0</v>
+      </c>
+      <c r="X9">
+        <v>0</v>
+      </c>
+      <c r="Y9">
+        <v>0</v>
+      </c>
+      <c r="Z9">
+        <v>0</v>
+      </c>
+      <c r="AA9">
+        <v>0</v>
+      </c>
+      <c r="AB9">
         <v>0</v>
       </c>
     </row>
@@ -816,10 +1222,10 @@
         <v>2</v>
       </c>
       <c r="G10">
-        <v>0.8511276216451236</v>
+        <v>0.8511271205223407</v>
       </c>
       <c r="H10">
-        <v>0.9834201131688234</v>
+        <v>0.9834195341555106</v>
       </c>
       <c r="I10">
         <v>0.8654771345916237</v>
@@ -837,6 +1243,48 @@
         <v>520</v>
       </c>
       <c r="N10">
+        <v>0</v>
+      </c>
+      <c r="O10">
+        <v>520</v>
+      </c>
+      <c r="P10">
+        <v>520</v>
+      </c>
+      <c r="Q10">
+        <v>0</v>
+      </c>
+      <c r="R10">
+        <v>0</v>
+      </c>
+      <c r="S10">
+        <v>0</v>
+      </c>
+      <c r="T10">
+        <v>0</v>
+      </c>
+      <c r="U10">
+        <v>0</v>
+      </c>
+      <c r="V10">
+        <v>0</v>
+      </c>
+      <c r="W10">
+        <v>0</v>
+      </c>
+      <c r="X10">
+        <v>0</v>
+      </c>
+      <c r="Y10">
+        <v>0</v>
+      </c>
+      <c r="Z10">
+        <v>0</v>
+      </c>
+      <c r="AA10">
+        <v>0</v>
+      </c>
+      <c r="AB10">
         <v>0</v>
       </c>
     </row>
@@ -862,13 +1310,13 @@
         <v>2</v>
       </c>
       <c r="G11">
-        <v>0.8482496899771208</v>
+        <v>0.8482492764943894</v>
       </c>
       <c r="H11">
-        <v>0.9836789163515479</v>
+        <v>0.983678436853294</v>
       </c>
       <c r="I11">
-        <v>0.8623237480002801</v>
+        <v>0.8623237480002802</v>
       </c>
       <c r="J11">
         <v>0.1356710618849967</v>
@@ -883,6 +1331,48 @@
         <v>520</v>
       </c>
       <c r="N11">
+        <v>0</v>
+      </c>
+      <c r="O11">
+        <v>520</v>
+      </c>
+      <c r="P11">
+        <v>520</v>
+      </c>
+      <c r="Q11">
+        <v>0</v>
+      </c>
+      <c r="R11">
+        <v>0</v>
+      </c>
+      <c r="S11">
+        <v>0</v>
+      </c>
+      <c r="T11">
+        <v>0</v>
+      </c>
+      <c r="U11">
+        <v>0</v>
+      </c>
+      <c r="V11">
+        <v>0</v>
+      </c>
+      <c r="W11">
+        <v>0</v>
+      </c>
+      <c r="X11">
+        <v>0</v>
+      </c>
+      <c r="Y11">
+        <v>0</v>
+      </c>
+      <c r="Z11">
+        <v>0</v>
+      </c>
+      <c r="AA11">
+        <v>0</v>
+      </c>
+      <c r="AB11">
         <v>0</v>
       </c>
     </row>
@@ -908,13 +1398,13 @@
         <v>2</v>
       </c>
       <c r="G12">
-        <v>0.8478978781244777</v>
+        <v>0.8478974969470973</v>
       </c>
       <c r="H12">
-        <v>0.9835761250497065</v>
+        <v>0.9835756828773879</v>
       </c>
       <c r="I12">
-        <v>0.8620561810420397</v>
+        <v>0.8620561810420396</v>
       </c>
       <c r="J12">
         <v>0.1357881844755813</v>
@@ -929,6 +1419,48 @@
         <v>520</v>
       </c>
       <c r="N12">
+        <v>0</v>
+      </c>
+      <c r="O12">
+        <v>520</v>
+      </c>
+      <c r="P12">
+        <v>520</v>
+      </c>
+      <c r="Q12">
+        <v>0</v>
+      </c>
+      <c r="R12">
+        <v>0</v>
+      </c>
+      <c r="S12">
+        <v>0</v>
+      </c>
+      <c r="T12">
+        <v>0</v>
+      </c>
+      <c r="U12">
+        <v>0</v>
+      </c>
+      <c r="V12">
+        <v>0</v>
+      </c>
+      <c r="W12">
+        <v>0</v>
+      </c>
+      <c r="X12">
+        <v>0</v>
+      </c>
+      <c r="Y12">
+        <v>0</v>
+      </c>
+      <c r="Z12">
+        <v>0</v>
+      </c>
+      <c r="AA12">
+        <v>0</v>
+      </c>
+      <c r="AB12">
         <v>0</v>
       </c>
     </row>
@@ -954,13 +1486,13 @@
         <v>2</v>
       </c>
       <c r="G13">
-        <v>0.8459624608526567</v>
+        <v>0.8459621148264678</v>
       </c>
       <c r="H13">
-        <v>0.9839658262464297</v>
+        <v>0.9839654237723715</v>
       </c>
       <c r="I13">
-        <v>0.8597478065674095</v>
+        <v>0.8597478065674093</v>
       </c>
       <c r="J13">
         <v>0.1367661341187663</v>
@@ -975,6 +1507,48 @@
         <v>520</v>
       </c>
       <c r="N13">
+        <v>0</v>
+      </c>
+      <c r="O13">
+        <v>520</v>
+      </c>
+      <c r="P13">
+        <v>520</v>
+      </c>
+      <c r="Q13">
+        <v>0</v>
+      </c>
+      <c r="R13">
+        <v>0</v>
+      </c>
+      <c r="S13">
+        <v>0</v>
+      </c>
+      <c r="T13">
+        <v>0</v>
+      </c>
+      <c r="U13">
+        <v>0</v>
+      </c>
+      <c r="V13">
+        <v>0</v>
+      </c>
+      <c r="W13">
+        <v>0</v>
+      </c>
+      <c r="X13">
+        <v>0</v>
+      </c>
+      <c r="Y13">
+        <v>0</v>
+      </c>
+      <c r="Z13">
+        <v>0</v>
+      </c>
+      <c r="AA13">
+        <v>0</v>
+      </c>
+      <c r="AB13">
         <v>0</v>
       </c>
     </row>
@@ -1000,10 +1574,10 @@
         <v>2</v>
       </c>
       <c r="G14">
-        <v>0.84545328143249</v>
+        <v>0.8454527605956127</v>
       </c>
       <c r="H14">
-        <v>0.9826350856293725</v>
+        <v>0.9826344802823939</v>
       </c>
       <c r="I14">
         <v>0.8603939486762593</v>
@@ -1021,6 +1595,48 @@
         <v>520</v>
       </c>
       <c r="N14">
+        <v>0</v>
+      </c>
+      <c r="O14">
+        <v>520</v>
+      </c>
+      <c r="P14">
+        <v>520</v>
+      </c>
+      <c r="Q14">
+        <v>0</v>
+      </c>
+      <c r="R14">
+        <v>0</v>
+      </c>
+      <c r="S14">
+        <v>0</v>
+      </c>
+      <c r="T14">
+        <v>0</v>
+      </c>
+      <c r="U14">
+        <v>0</v>
+      </c>
+      <c r="V14">
+        <v>0</v>
+      </c>
+      <c r="W14">
+        <v>0</v>
+      </c>
+      <c r="X14">
+        <v>0</v>
+      </c>
+      <c r="Y14">
+        <v>0</v>
+      </c>
+      <c r="Z14">
+        <v>0</v>
+      </c>
+      <c r="AA14">
+        <v>0</v>
+      </c>
+      <c r="AB14">
         <v>0</v>
       </c>
     </row>
@@ -1046,10 +1662,10 @@
         <v>2</v>
       </c>
       <c r="G15">
-        <v>0.8388644359806822</v>
+        <v>0.8388638825128004</v>
       </c>
       <c r="H15">
-        <v>0.9802712166982885</v>
+        <v>0.9802705699327201</v>
       </c>
       <c r="I15">
         <v>0.8557472888024936</v>
@@ -1067,6 +1683,48 @@
         <v>520</v>
       </c>
       <c r="N15">
+        <v>0</v>
+      </c>
+      <c r="O15">
+        <v>520</v>
+      </c>
+      <c r="P15">
+        <v>520</v>
+      </c>
+      <c r="Q15">
+        <v>0</v>
+      </c>
+      <c r="R15">
+        <v>0</v>
+      </c>
+      <c r="S15">
+        <v>0</v>
+      </c>
+      <c r="T15">
+        <v>0</v>
+      </c>
+      <c r="U15">
+        <v>0</v>
+      </c>
+      <c r="V15">
+        <v>0</v>
+      </c>
+      <c r="W15">
+        <v>0</v>
+      </c>
+      <c r="X15">
+        <v>0</v>
+      </c>
+      <c r="Y15">
+        <v>0</v>
+      </c>
+      <c r="Z15">
+        <v>0</v>
+      </c>
+      <c r="AA15">
+        <v>0</v>
+      </c>
+      <c r="AB15">
         <v>0</v>
       </c>
     </row>
@@ -1092,13 +1750,13 @@
         <v>2</v>
       </c>
       <c r="G16">
-        <v>0.8371262591108037</v>
+        <v>0.8371256120037543</v>
       </c>
       <c r="H16">
-        <v>0.9796065898451118</v>
+        <v>0.9796058325993285</v>
       </c>
       <c r="I16">
-        <v>0.8545535195339631</v>
+        <v>0.854553519533963</v>
       </c>
       <c r="J16">
         <v>0.1393632266132772</v>
@@ -1113,6 +1771,48 @@
         <v>520</v>
       </c>
       <c r="N16">
+        <v>0</v>
+      </c>
+      <c r="O16">
+        <v>520</v>
+      </c>
+      <c r="P16">
+        <v>520</v>
+      </c>
+      <c r="Q16">
+        <v>0</v>
+      </c>
+      <c r="R16">
+        <v>0</v>
+      </c>
+      <c r="S16">
+        <v>0</v>
+      </c>
+      <c r="T16">
+        <v>0</v>
+      </c>
+      <c r="U16">
+        <v>0</v>
+      </c>
+      <c r="V16">
+        <v>0</v>
+      </c>
+      <c r="W16">
+        <v>0</v>
+      </c>
+      <c r="X16">
+        <v>0</v>
+      </c>
+      <c r="Y16">
+        <v>0</v>
+      </c>
+      <c r="Z16">
+        <v>0</v>
+      </c>
+      <c r="AA16">
+        <v>0</v>
+      </c>
+      <c r="AB16">
         <v>0</v>
       </c>
     </row>
@@ -1138,13 +1838,13 @@
         <v>2</v>
       </c>
       <c r="G17">
-        <v>0.7196494052208635</v>
+        <v>0.7196489319286843</v>
       </c>
       <c r="H17">
-        <v>0.9542746945367271</v>
+        <v>0.9542740669384183</v>
       </c>
       <c r="I17">
-        <v>0.7541323366750625</v>
+        <v>0.7541323366750624</v>
       </c>
       <c r="J17">
         <v>0.1757318402802894</v>
@@ -1159,6 +1859,48 @@
         <v>520</v>
       </c>
       <c r="N17">
+        <v>0</v>
+      </c>
+      <c r="O17">
+        <v>520</v>
+      </c>
+      <c r="P17">
+        <v>520</v>
+      </c>
+      <c r="Q17">
+        <v>0</v>
+      </c>
+      <c r="R17">
+        <v>520</v>
+      </c>
+      <c r="S17">
+        <v>1</v>
+      </c>
+      <c r="T17">
+        <v>520</v>
+      </c>
+      <c r="U17">
+        <v>520</v>
+      </c>
+      <c r="V17">
+        <v>0</v>
+      </c>
+      <c r="W17">
+        <v>0</v>
+      </c>
+      <c r="X17">
+        <v>0</v>
+      </c>
+      <c r="Y17">
+        <v>520</v>
+      </c>
+      <c r="Z17">
+        <v>0</v>
+      </c>
+      <c r="AA17">
+        <v>0</v>
+      </c>
+      <c r="AB17">
         <v>0</v>
       </c>
     </row>
@@ -1184,10 +1926,10 @@
         <v>2</v>
       </c>
       <c r="G18">
-        <v>0.7176229410412458</v>
+        <v>0.7176222357716626</v>
       </c>
       <c r="H18">
-        <v>0.9496132741625081</v>
+        <v>0.9496123408961368</v>
       </c>
       <c r="I18">
         <v>0.7557001998251748</v>
@@ -1205,6 +1947,48 @@
         <v>520</v>
       </c>
       <c r="N18">
+        <v>0</v>
+      </c>
+      <c r="O18">
+        <v>520</v>
+      </c>
+      <c r="P18">
+        <v>520</v>
+      </c>
+      <c r="Q18">
+        <v>0</v>
+      </c>
+      <c r="R18">
+        <v>520</v>
+      </c>
+      <c r="S18">
+        <v>1</v>
+      </c>
+      <c r="T18">
+        <v>520</v>
+      </c>
+      <c r="U18">
+        <v>520</v>
+      </c>
+      <c r="V18">
+        <v>0</v>
+      </c>
+      <c r="W18">
+        <v>0</v>
+      </c>
+      <c r="X18">
+        <v>0</v>
+      </c>
+      <c r="Y18">
+        <v>520</v>
+      </c>
+      <c r="Z18">
+        <v>0</v>
+      </c>
+      <c r="AA18">
+        <v>0</v>
+      </c>
+      <c r="AB18">
         <v>0</v>
       </c>
     </row>
@@ -1230,10 +2014,10 @@
         <v>2</v>
       </c>
       <c r="G19">
-        <v>0.7169639027931974</v>
+        <v>0.7169632040812435</v>
       </c>
       <c r="H19">
-        <v>0.9508193100195969</v>
+        <v>0.9508183834055576</v>
       </c>
       <c r="I19">
         <v>0.7540485297657874</v>
@@ -1251,6 +2035,48 @@
         <v>520</v>
       </c>
       <c r="N19">
+        <v>0</v>
+      </c>
+      <c r="O19">
+        <v>520</v>
+      </c>
+      <c r="P19">
+        <v>520</v>
+      </c>
+      <c r="Q19">
+        <v>0</v>
+      </c>
+      <c r="R19">
+        <v>520</v>
+      </c>
+      <c r="S19">
+        <v>1</v>
+      </c>
+      <c r="T19">
+        <v>520</v>
+      </c>
+      <c r="U19">
+        <v>520</v>
+      </c>
+      <c r="V19">
+        <v>0</v>
+      </c>
+      <c r="W19">
+        <v>0</v>
+      </c>
+      <c r="X19">
+        <v>0</v>
+      </c>
+      <c r="Y19">
+        <v>520</v>
+      </c>
+      <c r="Z19">
+        <v>0</v>
+      </c>
+      <c r="AA19">
+        <v>0</v>
+      </c>
+      <c r="AB19">
         <v>0</v>
       </c>
     </row>
@@ -1276,13 +2102,13 @@
         <v>2</v>
       </c>
       <c r="G20">
-        <v>0.7149546667482524</v>
+        <v>0.7149541024912957</v>
       </c>
       <c r="H20">
-        <v>0.9508153645329895</v>
+        <v>0.9508146141299095</v>
       </c>
       <c r="I20">
-        <v>0.751938487131427</v>
+        <v>0.7519384871314269</v>
       </c>
       <c r="J20">
         <v>0.1764792327069223</v>
@@ -1297,6 +2123,48 @@
         <v>520</v>
       </c>
       <c r="N20">
+        <v>0</v>
+      </c>
+      <c r="O20">
+        <v>520</v>
+      </c>
+      <c r="P20">
+        <v>520</v>
+      </c>
+      <c r="Q20">
+        <v>0</v>
+      </c>
+      <c r="R20">
+        <v>520</v>
+      </c>
+      <c r="S20">
+        <v>1</v>
+      </c>
+      <c r="T20">
+        <v>520</v>
+      </c>
+      <c r="U20">
+        <v>520</v>
+      </c>
+      <c r="V20">
+        <v>0</v>
+      </c>
+      <c r="W20">
+        <v>0</v>
+      </c>
+      <c r="X20">
+        <v>0</v>
+      </c>
+      <c r="Y20">
+        <v>520</v>
+      </c>
+      <c r="Z20">
+        <v>0</v>
+      </c>
+      <c r="AA20">
+        <v>0</v>
+      </c>
+      <c r="AB20">
         <v>0</v>
       </c>
     </row>
@@ -1322,10 +2190,10 @@
         <v>2</v>
       </c>
       <c r="G21">
-        <v>0.6905879259543628</v>
+        <v>0.6905869946397264</v>
       </c>
       <c r="H21">
-        <v>0.9403388974336522</v>
+        <v>0.9403376293092823</v>
       </c>
       <c r="I21">
         <v>0.7344032325357347</v>
@@ -1343,6 +2211,48 @@
         <v>520</v>
       </c>
       <c r="N21">
+        <v>0</v>
+      </c>
+      <c r="O21">
+        <v>520</v>
+      </c>
+      <c r="P21">
+        <v>520</v>
+      </c>
+      <c r="Q21">
+        <v>0</v>
+      </c>
+      <c r="R21">
+        <v>520</v>
+      </c>
+      <c r="S21">
+        <v>1</v>
+      </c>
+      <c r="T21">
+        <v>520</v>
+      </c>
+      <c r="U21">
+        <v>520</v>
+      </c>
+      <c r="V21">
+        <v>0</v>
+      </c>
+      <c r="W21">
+        <v>0</v>
+      </c>
+      <c r="X21">
+        <v>0</v>
+      </c>
+      <c r="Y21">
+        <v>520</v>
+      </c>
+      <c r="Z21">
+        <v>0</v>
+      </c>
+      <c r="AA21">
+        <v>0</v>
+      </c>
+      <c r="AB21">
         <v>0</v>
       </c>
     </row>
@@ -1368,10 +2278,10 @@
         <v>2</v>
       </c>
       <c r="G22">
-        <v>0.6889634245481938</v>
+        <v>0.6889625452670983</v>
       </c>
       <c r="H22">
-        <v>0.941527963387948</v>
+        <v>0.9415267617744667</v>
       </c>
       <c r="I22">
         <v>0.7317503582889473</v>
@@ -1389,6 +2299,48 @@
         <v>520</v>
       </c>
       <c r="N22">
+        <v>0</v>
+      </c>
+      <c r="O22">
+        <v>520</v>
+      </c>
+      <c r="P22">
+        <v>520</v>
+      </c>
+      <c r="Q22">
+        <v>0</v>
+      </c>
+      <c r="R22">
+        <v>520</v>
+      </c>
+      <c r="S22">
+        <v>1</v>
+      </c>
+      <c r="T22">
+        <v>520</v>
+      </c>
+      <c r="U22">
+        <v>520</v>
+      </c>
+      <c r="V22">
+        <v>0</v>
+      </c>
+      <c r="W22">
+        <v>0</v>
+      </c>
+      <c r="X22">
+        <v>0</v>
+      </c>
+      <c r="Y22">
+        <v>520</v>
+      </c>
+      <c r="Z22">
+        <v>0</v>
+      </c>
+      <c r="AA22">
+        <v>0</v>
+      </c>
+      <c r="AB22">
         <v>0</v>
       </c>
     </row>
@@ -1414,19 +2366,19 @@
         <v>2</v>
       </c>
       <c r="G23">
-        <v>0.6671989080327384</v>
+        <v>0.66719757022741</v>
       </c>
       <c r="H23">
-        <v>0.9400304794925844</v>
+        <v>0.9400284583990497</v>
       </c>
       <c r="I23">
-        <v>0.709763058313687</v>
+        <v>0.7097631611746155</v>
       </c>
       <c r="J23">
-        <v>0.1886228070946772</v>
+        <v>0.1886227781733275</v>
       </c>
       <c r="K23">
-        <v>0.1558668900959172</v>
+        <v>0.1558668430052432</v>
       </c>
       <c r="L23">
         <v>520</v>
@@ -1435,6 +2387,48 @@
         <v>520</v>
       </c>
       <c r="N23">
+        <v>0</v>
+      </c>
+      <c r="O23">
+        <v>520</v>
+      </c>
+      <c r="P23">
+        <v>520</v>
+      </c>
+      <c r="Q23">
+        <v>0</v>
+      </c>
+      <c r="R23">
+        <v>520</v>
+      </c>
+      <c r="S23">
+        <v>1</v>
+      </c>
+      <c r="T23">
+        <v>520</v>
+      </c>
+      <c r="U23">
+        <v>520</v>
+      </c>
+      <c r="V23">
+        <v>0</v>
+      </c>
+      <c r="W23">
+        <v>0</v>
+      </c>
+      <c r="X23">
+        <v>0</v>
+      </c>
+      <c r="Y23">
+        <v>520</v>
+      </c>
+      <c r="Z23">
+        <v>0</v>
+      </c>
+      <c r="AA23">
+        <v>0</v>
+      </c>
+      <c r="AB23">
         <v>0</v>
       </c>
     </row>
@@ -1460,19 +2454,19 @@
         <v>2</v>
       </c>
       <c r="G24">
-        <v>0.6528324821544894</v>
+        <v>0.6528311341156038</v>
       </c>
       <c r="H24">
-        <v>0.9312152337416069</v>
+        <v>0.931213229881152</v>
       </c>
       <c r="I24">
-        <v>0.701054341144549</v>
+        <v>0.7010544021146721</v>
       </c>
       <c r="J24">
-        <v>0.1909923963229661</v>
+        <v>0.1909923820573538</v>
       </c>
       <c r="K24">
-        <v>0.1586933954469022</v>
+        <v>0.1586933829569199</v>
       </c>
       <c r="L24">
         <v>520</v>
@@ -1481,6 +2475,48 @@
         <v>520</v>
       </c>
       <c r="N24">
+        <v>0</v>
+      </c>
+      <c r="O24">
+        <v>520</v>
+      </c>
+      <c r="P24">
+        <v>520</v>
+      </c>
+      <c r="Q24">
+        <v>0</v>
+      </c>
+      <c r="R24">
+        <v>520</v>
+      </c>
+      <c r="S24">
+        <v>1</v>
+      </c>
+      <c r="T24">
+        <v>520</v>
+      </c>
+      <c r="U24">
+        <v>520</v>
+      </c>
+      <c r="V24">
+        <v>0</v>
+      </c>
+      <c r="W24">
+        <v>0</v>
+      </c>
+      <c r="X24">
+        <v>0</v>
+      </c>
+      <c r="Y24">
+        <v>520</v>
+      </c>
+      <c r="Z24">
+        <v>0</v>
+      </c>
+      <c r="AA24">
+        <v>0</v>
+      </c>
+      <c r="AB24">
         <v>0</v>
       </c>
     </row>
@@ -1506,19 +2542,19 @@
         <v>2</v>
       </c>
       <c r="G25">
-        <v>0.6512343721439366</v>
+        <v>0.6512330446620629</v>
       </c>
       <c r="H25">
-        <v>0.9318672205600289</v>
+        <v>0.9318652071301703</v>
       </c>
       <c r="I25">
-        <v>0.6988488893863667</v>
+        <v>0.6988489748078914</v>
       </c>
       <c r="J25">
-        <v>0.1915432813078952</v>
+        <v>0.1915432604149389</v>
       </c>
       <c r="K25">
-        <v>0.158639923465213</v>
+        <v>0.158639908657921</v>
       </c>
       <c r="L25">
         <v>520</v>
@@ -1527,6 +2563,48 @@
         <v>520</v>
       </c>
       <c r="N25">
+        <v>0</v>
+      </c>
+      <c r="O25">
+        <v>520</v>
+      </c>
+      <c r="P25">
+        <v>520</v>
+      </c>
+      <c r="Q25">
+        <v>0</v>
+      </c>
+      <c r="R25">
+        <v>520</v>
+      </c>
+      <c r="S25">
+        <v>1</v>
+      </c>
+      <c r="T25">
+        <v>520</v>
+      </c>
+      <c r="U25">
+        <v>520</v>
+      </c>
+      <c r="V25">
+        <v>0</v>
+      </c>
+      <c r="W25">
+        <v>0</v>
+      </c>
+      <c r="X25">
+        <v>0</v>
+      </c>
+      <c r="Y25">
+        <v>520</v>
+      </c>
+      <c r="Z25">
+        <v>0</v>
+      </c>
+      <c r="AA25">
+        <v>0</v>
+      </c>
+      <c r="AB25">
         <v>0</v>
       </c>
     </row>
@@ -1552,19 +2630,19 @@
         <v>2</v>
       </c>
       <c r="G26">
-        <v>0.6442620280414607</v>
+        <v>0.6442604886177106</v>
       </c>
       <c r="H26">
-        <v>0.9259120984346623</v>
+        <v>0.9259098932808812</v>
       </c>
       <c r="I26">
-        <v>0.6958133813465054</v>
+        <v>0.6958133758943102</v>
       </c>
       <c r="J26">
-        <v>0.1924196129580403</v>
+        <v>0.1924196140133874</v>
       </c>
       <c r="K26">
-        <v>0.1597804160401544</v>
+        <v>0.1597804180465117</v>
       </c>
       <c r="L26">
         <v>520</v>
@@ -1573,6 +2651,48 @@
         <v>520</v>
       </c>
       <c r="N26">
+        <v>0</v>
+      </c>
+      <c r="O26">
+        <v>520</v>
+      </c>
+      <c r="P26">
+        <v>520</v>
+      </c>
+      <c r="Q26">
+        <v>0</v>
+      </c>
+      <c r="R26">
+        <v>520</v>
+      </c>
+      <c r="S26">
+        <v>1</v>
+      </c>
+      <c r="T26">
+        <v>520</v>
+      </c>
+      <c r="U26">
+        <v>520</v>
+      </c>
+      <c r="V26">
+        <v>0</v>
+      </c>
+      <c r="W26">
+        <v>0</v>
+      </c>
+      <c r="X26">
+        <v>0</v>
+      </c>
+      <c r="Y26">
+        <v>520</v>
+      </c>
+      <c r="Z26">
+        <v>0</v>
+      </c>
+      <c r="AA26">
+        <v>0</v>
+      </c>
+      <c r="AB26">
         <v>0</v>
       </c>
     </row>
@@ -1598,19 +2718,19 @@
         <v>2</v>
       </c>
       <c r="G27">
-        <v>0.6359835392976639</v>
+        <v>0.6359820427152513</v>
       </c>
       <c r="H27">
-        <v>0.9197250956492555</v>
+        <v>0.9197229257017338</v>
       </c>
       <c r="I27">
-        <v>0.6914930801672953</v>
+        <v>0.6914930844308435</v>
       </c>
       <c r="J27">
-        <v>0.1935887721193069</v>
+        <v>0.1935887711224843</v>
       </c>
       <c r="K27">
-        <v>0.1606782285886126</v>
+        <v>0.1606782285375603</v>
       </c>
       <c r="L27">
         <v>520</v>
@@ -1619,6 +2739,48 @@
         <v>520</v>
       </c>
       <c r="N27">
+        <v>0</v>
+      </c>
+      <c r="O27">
+        <v>520</v>
+      </c>
+      <c r="P27">
+        <v>520</v>
+      </c>
+      <c r="Q27">
+        <v>0</v>
+      </c>
+      <c r="R27">
+        <v>520</v>
+      </c>
+      <c r="S27">
+        <v>1</v>
+      </c>
+      <c r="T27">
+        <v>520</v>
+      </c>
+      <c r="U27">
+        <v>520</v>
+      </c>
+      <c r="V27">
+        <v>0</v>
+      </c>
+      <c r="W27">
+        <v>0</v>
+      </c>
+      <c r="X27">
+        <v>0</v>
+      </c>
+      <c r="Y27">
+        <v>520</v>
+      </c>
+      <c r="Z27">
+        <v>0</v>
+      </c>
+      <c r="AA27">
+        <v>0</v>
+      </c>
+      <c r="AB27">
         <v>0</v>
       </c>
     </row>
@@ -1644,19 +2806,19 @@
         <v>2</v>
       </c>
       <c r="G28">
-        <v>0.6305803700532067</v>
+        <v>0.6305787285007819</v>
       </c>
       <c r="H28">
-        <v>0.9155409866715644</v>
+        <v>0.9155385914288812</v>
       </c>
       <c r="I28">
-        <v>0.6887516552870803</v>
+        <v>0.6887516642161829</v>
       </c>
       <c r="J28">
-        <v>0.1943716319959523</v>
+        <v>0.1943716299172568</v>
       </c>
       <c r="K28">
-        <v>0.1604890017758653</v>
+        <v>0.1604889982098709</v>
       </c>
       <c r="L28">
         <v>520</v>
@@ -1665,6 +2827,48 @@
         <v>520</v>
       </c>
       <c r="N28">
+        <v>0</v>
+      </c>
+      <c r="O28">
+        <v>520</v>
+      </c>
+      <c r="P28">
+        <v>520</v>
+      </c>
+      <c r="Q28">
+        <v>0</v>
+      </c>
+      <c r="R28">
+        <v>520</v>
+      </c>
+      <c r="S28">
+        <v>1</v>
+      </c>
+      <c r="T28">
+        <v>520</v>
+      </c>
+      <c r="U28">
+        <v>520</v>
+      </c>
+      <c r="V28">
+        <v>0</v>
+      </c>
+      <c r="W28">
+        <v>0</v>
+      </c>
+      <c r="X28">
+        <v>0</v>
+      </c>
+      <c r="Y28">
+        <v>520</v>
+      </c>
+      <c r="Z28">
+        <v>0</v>
+      </c>
+      <c r="AA28">
+        <v>0</v>
+      </c>
+      <c r="AB28">
         <v>0</v>
       </c>
     </row>
@@ -1690,10 +2894,10 @@
         <v>1</v>
       </c>
       <c r="G29">
-        <v>0.5467478717072874</v>
+        <v>0.5467469030659569</v>
       </c>
       <c r="H29">
-        <v>0.8854276009611486</v>
+        <v>0.8854260323006857</v>
       </c>
       <c r="I29">
         <v>0.6174958529797153</v>
@@ -1711,6 +2915,48 @@
         <v>520</v>
       </c>
       <c r="N29">
+        <v>0</v>
+      </c>
+      <c r="O29">
+        <v>520</v>
+      </c>
+      <c r="P29">
+        <v>520</v>
+      </c>
+      <c r="Q29">
+        <v>0</v>
+      </c>
+      <c r="R29">
+        <v>0</v>
+      </c>
+      <c r="S29">
+        <v>0</v>
+      </c>
+      <c r="T29">
+        <v>0</v>
+      </c>
+      <c r="U29">
+        <v>0</v>
+      </c>
+      <c r="V29">
+        <v>0</v>
+      </c>
+      <c r="W29">
+        <v>0</v>
+      </c>
+      <c r="X29">
+        <v>0</v>
+      </c>
+      <c r="Y29">
+        <v>0</v>
+      </c>
+      <c r="Z29">
+        <v>0</v>
+      </c>
+      <c r="AA29">
+        <v>0</v>
+      </c>
+      <c r="AB29">
         <v>0</v>
       </c>
     </row>
@@ -1736,13 +2982,13 @@
         <v>1</v>
       </c>
       <c r="G30">
-        <v>0.5463507619816133</v>
+        <v>0.5463497234813487</v>
       </c>
       <c r="H30">
-        <v>0.8818102083370936</v>
+        <v>0.8818085321975173</v>
       </c>
       <c r="I30">
-        <v>0.6195786313382724</v>
+        <v>0.6195786313382723</v>
       </c>
       <c r="J30">
         <v>0.210118622666713</v>
@@ -1757,6 +3003,48 @@
         <v>520</v>
       </c>
       <c r="N30">
+        <v>0</v>
+      </c>
+      <c r="O30">
+        <v>520</v>
+      </c>
+      <c r="P30">
+        <v>520</v>
+      </c>
+      <c r="Q30">
+        <v>0</v>
+      </c>
+      <c r="R30">
+        <v>0</v>
+      </c>
+      <c r="S30">
+        <v>0</v>
+      </c>
+      <c r="T30">
+        <v>0</v>
+      </c>
+      <c r="U30">
+        <v>0</v>
+      </c>
+      <c r="V30">
+        <v>0</v>
+      </c>
+      <c r="W30">
+        <v>0</v>
+      </c>
+      <c r="X30">
+        <v>0</v>
+      </c>
+      <c r="Y30">
+        <v>0</v>
+      </c>
+      <c r="Z30">
+        <v>0</v>
+      </c>
+      <c r="AA30">
+        <v>0</v>
+      </c>
+      <c r="AB30">
         <v>0</v>
       </c>
     </row>
@@ -1782,13 +3070,13 @@
         <v>1</v>
       </c>
       <c r="G31">
-        <v>0.5441867863344318</v>
+        <v>0.5441859314192204</v>
       </c>
       <c r="H31">
-        <v>0.8880569900285936</v>
+        <v>0.8880555948947013</v>
       </c>
       <c r="I31">
-        <v>0.6127836303804221</v>
+        <v>0.6127836303804219</v>
       </c>
       <c r="J31">
         <v>0.2114399943011605</v>
@@ -1803,6 +3091,48 @@
         <v>520</v>
       </c>
       <c r="N31">
+        <v>0</v>
+      </c>
+      <c r="O31">
+        <v>520</v>
+      </c>
+      <c r="P31">
+        <v>520</v>
+      </c>
+      <c r="Q31">
+        <v>0</v>
+      </c>
+      <c r="R31">
+        <v>0</v>
+      </c>
+      <c r="S31">
+        <v>0</v>
+      </c>
+      <c r="T31">
+        <v>0</v>
+      </c>
+      <c r="U31">
+        <v>0</v>
+      </c>
+      <c r="V31">
+        <v>0</v>
+      </c>
+      <c r="W31">
+        <v>0</v>
+      </c>
+      <c r="X31">
+        <v>0</v>
+      </c>
+      <c r="Y31">
+        <v>0</v>
+      </c>
+      <c r="Z31">
+        <v>0</v>
+      </c>
+      <c r="AA31">
+        <v>0</v>
+      </c>
+      <c r="AB31">
         <v>0</v>
       </c>
     </row>
@@ -1828,13 +3158,13 @@
         <v>1</v>
       </c>
       <c r="G32">
-        <v>0.5440915465688648</v>
+        <v>0.5440905267547507</v>
       </c>
       <c r="H32">
-        <v>0.8840045605993925</v>
+        <v>0.8840029036717422</v>
       </c>
       <c r="I32">
-        <v>0.6154849995343324</v>
+        <v>0.6154849995343323</v>
       </c>
       <c r="J32">
         <v>0.2109359457670249</v>
@@ -1849,6 +3179,48 @@
         <v>520</v>
       </c>
       <c r="N32">
+        <v>0</v>
+      </c>
+      <c r="O32">
+        <v>520</v>
+      </c>
+      <c r="P32">
+        <v>520</v>
+      </c>
+      <c r="Q32">
+        <v>0</v>
+      </c>
+      <c r="R32">
+        <v>0</v>
+      </c>
+      <c r="S32">
+        <v>0</v>
+      </c>
+      <c r="T32">
+        <v>0</v>
+      </c>
+      <c r="U32">
+        <v>0</v>
+      </c>
+      <c r="V32">
+        <v>0</v>
+      </c>
+      <c r="W32">
+        <v>0</v>
+      </c>
+      <c r="X32">
+        <v>0</v>
+      </c>
+      <c r="Y32">
+        <v>0</v>
+      </c>
+      <c r="Z32">
+        <v>0</v>
+      </c>
+      <c r="AA32">
+        <v>0</v>
+      </c>
+      <c r="AB32">
         <v>0</v>
       </c>
     </row>
@@ -1874,13 +3246,13 @@
         <v>1</v>
       </c>
       <c r="G33">
-        <v>0.5427505120229421</v>
+        <v>0.5427495331834251</v>
       </c>
       <c r="H33">
-        <v>0.8820455743623908</v>
+        <v>0.8820439836111251</v>
       </c>
       <c r="I33">
-        <v>0.6153315971402987</v>
+        <v>0.6153315971402988</v>
       </c>
       <c r="J33">
         <v>0.2109711399074354</v>
@@ -1895,6 +3267,48 @@
         <v>520</v>
       </c>
       <c r="N33">
+        <v>0</v>
+      </c>
+      <c r="O33">
+        <v>520</v>
+      </c>
+      <c r="P33">
+        <v>520</v>
+      </c>
+      <c r="Q33">
+        <v>0</v>
+      </c>
+      <c r="R33">
+        <v>0</v>
+      </c>
+      <c r="S33">
+        <v>0</v>
+      </c>
+      <c r="T33">
+        <v>0</v>
+      </c>
+      <c r="U33">
+        <v>0</v>
+      </c>
+      <c r="V33">
+        <v>0</v>
+      </c>
+      <c r="W33">
+        <v>0</v>
+      </c>
+      <c r="X33">
+        <v>0</v>
+      </c>
+      <c r="Y33">
+        <v>0</v>
+      </c>
+      <c r="Z33">
+        <v>0</v>
+      </c>
+      <c r="AA33">
+        <v>0</v>
+      </c>
+      <c r="AB33">
         <v>0</v>
       </c>
     </row>
@@ -1920,10 +3334,10 @@
         <v>1</v>
       </c>
       <c r="G34">
-        <v>0.542656523389252</v>
+        <v>0.5426556683909164</v>
       </c>
       <c r="H34">
-        <v>0.8856304518764206</v>
+        <v>0.8856290564954943</v>
       </c>
       <c r="I34">
         <v>0.612734715974935</v>
@@ -1941,6 +3355,48 @@
         <v>520</v>
       </c>
       <c r="N34">
+        <v>0</v>
+      </c>
+      <c r="O34">
+        <v>520</v>
+      </c>
+      <c r="P34">
+        <v>520</v>
+      </c>
+      <c r="Q34">
+        <v>0</v>
+      </c>
+      <c r="R34">
+        <v>0</v>
+      </c>
+      <c r="S34">
+        <v>0</v>
+      </c>
+      <c r="T34">
+        <v>0</v>
+      </c>
+      <c r="U34">
+        <v>0</v>
+      </c>
+      <c r="V34">
+        <v>0</v>
+      </c>
+      <c r="W34">
+        <v>0</v>
+      </c>
+      <c r="X34">
+        <v>0</v>
+      </c>
+      <c r="Y34">
+        <v>0</v>
+      </c>
+      <c r="Z34">
+        <v>0</v>
+      </c>
+      <c r="AA34">
+        <v>0</v>
+      </c>
+      <c r="AB34">
         <v>0</v>
       </c>
     </row>
@@ -1966,13 +3422,13 @@
         <v>1</v>
       </c>
       <c r="G35">
-        <v>0.5399217050036177</v>
+        <v>0.5399201475986962</v>
       </c>
       <c r="H35">
-        <v>0.874234105480343</v>
+        <v>0.8742315837508298</v>
       </c>
       <c r="I35">
-        <v>0.6175939620966409</v>
+        <v>0.6175939620966407</v>
       </c>
       <c r="J35">
         <v>0.2107151639103583</v>
@@ -1987,6 +3443,48 @@
         <v>520</v>
       </c>
       <c r="N35">
+        <v>0</v>
+      </c>
+      <c r="O35">
+        <v>520</v>
+      </c>
+      <c r="P35">
+        <v>520</v>
+      </c>
+      <c r="Q35">
+        <v>0</v>
+      </c>
+      <c r="R35">
+        <v>0</v>
+      </c>
+      <c r="S35">
+        <v>0</v>
+      </c>
+      <c r="T35">
+        <v>0</v>
+      </c>
+      <c r="U35">
+        <v>0</v>
+      </c>
+      <c r="V35">
+        <v>0</v>
+      </c>
+      <c r="W35">
+        <v>0</v>
+      </c>
+      <c r="X35">
+        <v>0</v>
+      </c>
+      <c r="Y35">
+        <v>0</v>
+      </c>
+      <c r="Z35">
+        <v>0</v>
+      </c>
+      <c r="AA35">
+        <v>0</v>
+      </c>
+      <c r="AB35">
         <v>0</v>
       </c>
     </row>
@@ -2012,10 +3510,10 @@
         <v>1</v>
       </c>
       <c r="G36">
-        <v>0.5379808886934042</v>
+        <v>0.5379799465380435</v>
       </c>
       <c r="H36">
-        <v>0.873984773635388</v>
+        <v>0.8739832430430249</v>
       </c>
       <c r="I36">
         <v>0.6155494980257413</v>
@@ -2033,6 +3531,48 @@
         <v>520</v>
       </c>
       <c r="N36">
+        <v>0</v>
+      </c>
+      <c r="O36">
+        <v>520</v>
+      </c>
+      <c r="P36">
+        <v>520</v>
+      </c>
+      <c r="Q36">
+        <v>0</v>
+      </c>
+      <c r="R36">
+        <v>0</v>
+      </c>
+      <c r="S36">
+        <v>0</v>
+      </c>
+      <c r="T36">
+        <v>0</v>
+      </c>
+      <c r="U36">
+        <v>0</v>
+      </c>
+      <c r="V36">
+        <v>0</v>
+      </c>
+      <c r="W36">
+        <v>0</v>
+      </c>
+      <c r="X36">
+        <v>0</v>
+      </c>
+      <c r="Y36">
+        <v>0</v>
+      </c>
+      <c r="Z36">
+        <v>0</v>
+      </c>
+      <c r="AA36">
+        <v>0</v>
+      </c>
+      <c r="AB36">
         <v>0</v>
       </c>
     </row>
@@ -2058,10 +3598,10 @@
         <v>1</v>
       </c>
       <c r="G37">
-        <v>0.5361067477414744</v>
+        <v>0.5361057779822851</v>
       </c>
       <c r="H37">
-        <v>0.876921072866553</v>
+        <v>0.8769194866110689</v>
       </c>
       <c r="I37">
         <v>0.6113511971938407</v>
@@ -2079,6 +3619,48 @@
         <v>520</v>
       </c>
       <c r="N37">
+        <v>0</v>
+      </c>
+      <c r="O37">
+        <v>520</v>
+      </c>
+      <c r="P37">
+        <v>520</v>
+      </c>
+      <c r="Q37">
+        <v>0</v>
+      </c>
+      <c r="R37">
+        <v>0</v>
+      </c>
+      <c r="S37">
+        <v>0</v>
+      </c>
+      <c r="T37">
+        <v>0</v>
+      </c>
+      <c r="U37">
+        <v>0</v>
+      </c>
+      <c r="V37">
+        <v>0</v>
+      </c>
+      <c r="W37">
+        <v>0</v>
+      </c>
+      <c r="X37">
+        <v>0</v>
+      </c>
+      <c r="Y37">
+        <v>0</v>
+      </c>
+      <c r="Z37">
+        <v>0</v>
+      </c>
+      <c r="AA37">
+        <v>0</v>
+      </c>
+      <c r="AB37">
         <v>0</v>
       </c>
     </row>
@@ -2104,10 +3686,10 @@
         <v>1</v>
       </c>
       <c r="G38">
-        <v>0.5355173643955184</v>
+        <v>0.5355164395611555</v>
       </c>
       <c r="H38">
-        <v>0.8745300746300552</v>
+        <v>0.8745285643233532</v>
       </c>
       <c r="I38">
         <v>0.6123487115317946</v>
@@ -2125,6 +3707,48 @@
         <v>520</v>
       </c>
       <c r="N38">
+        <v>0</v>
+      </c>
+      <c r="O38">
+        <v>520</v>
+      </c>
+      <c r="P38">
+        <v>520</v>
+      </c>
+      <c r="Q38">
+        <v>0</v>
+      </c>
+      <c r="R38">
+        <v>0</v>
+      </c>
+      <c r="S38">
+        <v>0</v>
+      </c>
+      <c r="T38">
+        <v>0</v>
+      </c>
+      <c r="U38">
+        <v>0</v>
+      </c>
+      <c r="V38">
+        <v>0</v>
+      </c>
+      <c r="W38">
+        <v>0</v>
+      </c>
+      <c r="X38">
+        <v>0</v>
+      </c>
+      <c r="Y38">
+        <v>0</v>
+      </c>
+      <c r="Z38">
+        <v>0</v>
+      </c>
+      <c r="AA38">
+        <v>0</v>
+      </c>
+      <c r="AB38">
         <v>0</v>
       </c>
     </row>
@@ -2150,10 +3774,10 @@
         <v>1</v>
       </c>
       <c r="G39">
-        <v>0.53215566810695</v>
+        <v>0.5321542318159114</v>
       </c>
       <c r="H39">
-        <v>0.868134679407209</v>
+        <v>0.868132336306994</v>
       </c>
       <c r="I39">
         <v>0.6129874554375866</v>
@@ -2171,6 +3795,48 @@
         <v>520</v>
       </c>
       <c r="N39">
+        <v>0</v>
+      </c>
+      <c r="O39">
+        <v>520</v>
+      </c>
+      <c r="P39">
+        <v>520</v>
+      </c>
+      <c r="Q39">
+        <v>0</v>
+      </c>
+      <c r="R39">
+        <v>0</v>
+      </c>
+      <c r="S39">
+        <v>0</v>
+      </c>
+      <c r="T39">
+        <v>0</v>
+      </c>
+      <c r="U39">
+        <v>0</v>
+      </c>
+      <c r="V39">
+        <v>0</v>
+      </c>
+      <c r="W39">
+        <v>0</v>
+      </c>
+      <c r="X39">
+        <v>0</v>
+      </c>
+      <c r="Y39">
+        <v>0</v>
+      </c>
+      <c r="Z39">
+        <v>0</v>
+      </c>
+      <c r="AA39">
+        <v>0</v>
+      </c>
+      <c r="AB39">
         <v>0</v>
       </c>
     </row>
@@ -2196,10 +3862,10 @@
         <v>1</v>
       </c>
       <c r="G40">
-        <v>0.5209965049382318</v>
+        <v>0.5209950066213321</v>
       </c>
       <c r="H40">
-        <v>0.8592861781274166</v>
+        <v>0.859283706934251</v>
       </c>
       <c r="I40">
         <v>0.6063131447937447</v>
@@ -2217,6 +3883,48 @@
         <v>520</v>
       </c>
       <c r="N40">
+        <v>0</v>
+      </c>
+      <c r="O40">
+        <v>520</v>
+      </c>
+      <c r="P40">
+        <v>520</v>
+      </c>
+      <c r="Q40">
+        <v>0</v>
+      </c>
+      <c r="R40">
+        <v>0</v>
+      </c>
+      <c r="S40">
+        <v>0</v>
+      </c>
+      <c r="T40">
+        <v>0</v>
+      </c>
+      <c r="U40">
+        <v>0</v>
+      </c>
+      <c r="V40">
+        <v>0</v>
+      </c>
+      <c r="W40">
+        <v>0</v>
+      </c>
+      <c r="X40">
+        <v>0</v>
+      </c>
+      <c r="Y40">
+        <v>0</v>
+      </c>
+      <c r="Z40">
+        <v>0</v>
+      </c>
+      <c r="AA40">
+        <v>0</v>
+      </c>
+      <c r="AB40">
         <v>0</v>
       </c>
     </row>
@@ -2242,10 +3950,10 @@
         <v>1</v>
       </c>
       <c r="G41">
-        <v>0.5209811611297677</v>
+        <v>0.5209795549793105</v>
       </c>
       <c r="H41">
-        <v>0.8538295370907151</v>
+        <v>0.8538269047907326</v>
       </c>
       <c r="I41">
         <v>0.6101699911962826</v>
@@ -2263,6 +3971,48 @@
         <v>520</v>
       </c>
       <c r="N41">
+        <v>0</v>
+      </c>
+      <c r="O41">
+        <v>520</v>
+      </c>
+      <c r="P41">
+        <v>520</v>
+      </c>
+      <c r="Q41">
+        <v>0</v>
+      </c>
+      <c r="R41">
+        <v>0</v>
+      </c>
+      <c r="S41">
+        <v>0</v>
+      </c>
+      <c r="T41">
+        <v>0</v>
+      </c>
+      <c r="U41">
+        <v>0</v>
+      </c>
+      <c r="V41">
+        <v>0</v>
+      </c>
+      <c r="W41">
+        <v>0</v>
+      </c>
+      <c r="X41">
+        <v>0</v>
+      </c>
+      <c r="Y41">
+        <v>0</v>
+      </c>
+      <c r="Z41">
+        <v>0</v>
+      </c>
+      <c r="AA41">
+        <v>0</v>
+      </c>
+      <c r="AB41">
         <v>0</v>
       </c>
     </row>
@@ -2288,10 +4038,10 @@
         <v>1</v>
       </c>
       <c r="G42">
-        <v>0.518355464839952</v>
+        <v>0.5183539453322357</v>
       </c>
       <c r="H42">
-        <v>0.8557598125671003</v>
+        <v>0.8557573039919494</v>
       </c>
       <c r="I42">
         <v>0.6057254117659417</v>
@@ -2309,6 +4059,48 @@
         <v>520</v>
       </c>
       <c r="N42">
+        <v>0</v>
+      </c>
+      <c r="O42">
+        <v>520</v>
+      </c>
+      <c r="P42">
+        <v>520</v>
+      </c>
+      <c r="Q42">
+        <v>0</v>
+      </c>
+      <c r="R42">
+        <v>0</v>
+      </c>
+      <c r="S42">
+        <v>0</v>
+      </c>
+      <c r="T42">
+        <v>0</v>
+      </c>
+      <c r="U42">
+        <v>0</v>
+      </c>
+      <c r="V42">
+        <v>0</v>
+      </c>
+      <c r="W42">
+        <v>0</v>
+      </c>
+      <c r="X42">
+        <v>0</v>
+      </c>
+      <c r="Y42">
+        <v>0</v>
+      </c>
+      <c r="Z42">
+        <v>0</v>
+      </c>
+      <c r="AA42">
+        <v>0</v>
+      </c>
+      <c r="AB42">
         <v>0</v>
       </c>
     </row>
@@ -2334,10 +4126,10 @@
         <v>1</v>
       </c>
       <c r="G43">
-        <v>0.5183030319514151</v>
+        <v>0.518301381810877</v>
       </c>
       <c r="H43">
-        <v>0.8504911815996964</v>
+        <v>0.8504884738594566</v>
       </c>
       <c r="I43">
         <v>0.6094161152576966</v>
@@ -2355,6 +4147,48 @@
         <v>520</v>
       </c>
       <c r="N43">
+        <v>0</v>
+      </c>
+      <c r="O43">
+        <v>520</v>
+      </c>
+      <c r="P43">
+        <v>520</v>
+      </c>
+      <c r="Q43">
+        <v>0</v>
+      </c>
+      <c r="R43">
+        <v>0</v>
+      </c>
+      <c r="S43">
+        <v>0</v>
+      </c>
+      <c r="T43">
+        <v>0</v>
+      </c>
+      <c r="U43">
+        <v>0</v>
+      </c>
+      <c r="V43">
+        <v>0</v>
+      </c>
+      <c r="W43">
+        <v>0</v>
+      </c>
+      <c r="X43">
+        <v>0</v>
+      </c>
+      <c r="Y43">
+        <v>0</v>
+      </c>
+      <c r="Z43">
+        <v>0</v>
+      </c>
+      <c r="AA43">
+        <v>0</v>
+      </c>
+      <c r="AB43">
         <v>0</v>
       </c>
     </row>
@@ -2380,13 +4214,13 @@
         <v>1</v>
       </c>
       <c r="G44">
-        <v>0.5144409991717317</v>
+        <v>0.5144393273657739</v>
       </c>
       <c r="H44">
-        <v>0.8495701624638864</v>
+        <v>0.8495674015710699</v>
       </c>
       <c r="I44">
-        <v>0.6055309165752388</v>
+        <v>0.6055309165752387</v>
       </c>
       <c r="J44">
         <v>0.2134890528083476</v>
@@ -2401,6 +4235,48 @@
         <v>520</v>
       </c>
       <c r="N44">
+        <v>0</v>
+      </c>
+      <c r="O44">
+        <v>520</v>
+      </c>
+      <c r="P44">
+        <v>520</v>
+      </c>
+      <c r="Q44">
+        <v>0</v>
+      </c>
+      <c r="R44">
+        <v>0</v>
+      </c>
+      <c r="S44">
+        <v>0</v>
+      </c>
+      <c r="T44">
+        <v>0</v>
+      </c>
+      <c r="U44">
+        <v>0</v>
+      </c>
+      <c r="V44">
+        <v>0</v>
+      </c>
+      <c r="W44">
+        <v>0</v>
+      </c>
+      <c r="X44">
+        <v>0</v>
+      </c>
+      <c r="Y44">
+        <v>0</v>
+      </c>
+      <c r="Z44">
+        <v>0</v>
+      </c>
+      <c r="AA44">
+        <v>0</v>
+      </c>
+      <c r="AB44">
         <v>0</v>
       </c>
     </row>
@@ -2426,10 +4302,10 @@
         <v>1</v>
       </c>
       <c r="G45">
-        <v>0.5061867693872224</v>
+        <v>0.5061850333805495</v>
       </c>
       <c r="H45">
-        <v>0.8409331129220113</v>
+        <v>0.8409302288768649</v>
       </c>
       <c r="I45">
         <v>0.6019346385687711</v>
@@ -2447,6 +4323,48 @@
         <v>520</v>
       </c>
       <c r="N45">
+        <v>0</v>
+      </c>
+      <c r="O45">
+        <v>520</v>
+      </c>
+      <c r="P45">
+        <v>520</v>
+      </c>
+      <c r="Q45">
+        <v>0</v>
+      </c>
+      <c r="R45">
+        <v>0</v>
+      </c>
+      <c r="S45">
+        <v>0</v>
+      </c>
+      <c r="T45">
+        <v>0</v>
+      </c>
+      <c r="U45">
+        <v>0</v>
+      </c>
+      <c r="V45">
+        <v>0</v>
+      </c>
+      <c r="W45">
+        <v>0</v>
+      </c>
+      <c r="X45">
+        <v>0</v>
+      </c>
+      <c r="Y45">
+        <v>0</v>
+      </c>
+      <c r="Z45">
+        <v>0</v>
+      </c>
+      <c r="AA45">
+        <v>0</v>
+      </c>
+      <c r="AB45">
         <v>0</v>
       </c>
     </row>
@@ -2472,10 +4390,10 @@
         <v>1</v>
       </c>
       <c r="G46">
-        <v>0.5035206229038333</v>
+        <v>0.5035189333500776</v>
       </c>
       <c r="H46">
-        <v>0.8408304629756794</v>
+        <v>0.8408276415852496</v>
       </c>
       <c r="I46">
         <v>0.5988372746651989</v>
@@ -2493,6 +4411,48 @@
         <v>520</v>
       </c>
       <c r="N46">
+        <v>0</v>
+      </c>
+      <c r="O46">
+        <v>520</v>
+      </c>
+      <c r="P46">
+        <v>520</v>
+      </c>
+      <c r="Q46">
+        <v>0</v>
+      </c>
+      <c r="R46">
+        <v>0</v>
+      </c>
+      <c r="S46">
+        <v>0</v>
+      </c>
+      <c r="T46">
+        <v>0</v>
+      </c>
+      <c r="U46">
+        <v>0</v>
+      </c>
+      <c r="V46">
+        <v>0</v>
+      </c>
+      <c r="W46">
+        <v>0</v>
+      </c>
+      <c r="X46">
+        <v>0</v>
+      </c>
+      <c r="Y46">
+        <v>0</v>
+      </c>
+      <c r="Z46">
+        <v>0</v>
+      </c>
+      <c r="AA46">
+        <v>0</v>
+      </c>
+      <c r="AB46">
         <v>0</v>
       </c>
     </row>
@@ -2518,13 +4478,13 @@
         <v>1</v>
       </c>
       <c r="G47">
-        <v>0.2450381075213826</v>
+        <v>0.2450375005707693</v>
       </c>
       <c r="H47">
-        <v>0.6688372488477236</v>
+        <v>0.6688355921618208</v>
       </c>
       <c r="I47">
-        <v>0.3663643254671232</v>
+        <v>0.3663643254671231</v>
       </c>
       <c r="J47">
         <v>0.2489908502028701</v>
@@ -2539,6 +4499,48 @@
         <v>520</v>
       </c>
       <c r="N47">
+        <v>0</v>
+      </c>
+      <c r="O47">
+        <v>520</v>
+      </c>
+      <c r="P47">
+        <v>520</v>
+      </c>
+      <c r="Q47">
+        <v>0</v>
+      </c>
+      <c r="R47">
+        <v>520</v>
+      </c>
+      <c r="S47">
+        <v>1</v>
+      </c>
+      <c r="T47">
+        <v>520</v>
+      </c>
+      <c r="U47">
+        <v>520</v>
+      </c>
+      <c r="V47">
+        <v>0</v>
+      </c>
+      <c r="W47">
+        <v>0</v>
+      </c>
+      <c r="X47">
+        <v>0</v>
+      </c>
+      <c r="Y47">
+        <v>520</v>
+      </c>
+      <c r="Z47">
+        <v>0</v>
+      </c>
+      <c r="AA47">
+        <v>0</v>
+      </c>
+      <c r="AB47">
         <v>0</v>
       </c>
     </row>
@@ -2564,10 +4566,10 @@
         <v>1</v>
       </c>
       <c r="G48">
-        <v>0.2255559178913771</v>
+        <v>0.2255553133808242</v>
       </c>
       <c r="H48">
-        <v>0.6399244709804067</v>
+        <v>0.6399227559241164</v>
       </c>
       <c r="I48">
         <v>0.3524727184534927</v>
@@ -2585,6 +4587,48 @@
         <v>520</v>
       </c>
       <c r="N48">
+        <v>0</v>
+      </c>
+      <c r="O48">
+        <v>520</v>
+      </c>
+      <c r="P48">
+        <v>520</v>
+      </c>
+      <c r="Q48">
+        <v>0</v>
+      </c>
+      <c r="R48">
+        <v>520</v>
+      </c>
+      <c r="S48">
+        <v>1</v>
+      </c>
+      <c r="T48">
+        <v>520</v>
+      </c>
+      <c r="U48">
+        <v>520</v>
+      </c>
+      <c r="V48">
+        <v>0</v>
+      </c>
+      <c r="W48">
+        <v>0</v>
+      </c>
+      <c r="X48">
+        <v>0</v>
+      </c>
+      <c r="Y48">
+        <v>520</v>
+      </c>
+      <c r="Z48">
+        <v>0</v>
+      </c>
+      <c r="AA48">
+        <v>0</v>
+      </c>
+      <c r="AB48">
         <v>0</v>
       </c>
     </row>
@@ -2610,13 +4654,13 @@
         <v>1</v>
       </c>
       <c r="G49">
-        <v>0.2236193308978556</v>
+        <v>0.2236187384142684</v>
       </c>
       <c r="H49">
-        <v>0.6415246810986615</v>
+        <v>0.6415229813670561</v>
       </c>
       <c r="I49">
-        <v>0.3485747898504698</v>
+        <v>0.3485747898504697</v>
       </c>
       <c r="J49">
         <v>0.2508076597938882</v>
@@ -2631,6 +4675,48 @@
         <v>520</v>
       </c>
       <c r="N49">
+        <v>0</v>
+      </c>
+      <c r="O49">
+        <v>520</v>
+      </c>
+      <c r="P49">
+        <v>520</v>
+      </c>
+      <c r="Q49">
+        <v>0</v>
+      </c>
+      <c r="R49">
+        <v>520</v>
+      </c>
+      <c r="S49">
+        <v>1</v>
+      </c>
+      <c r="T49">
+        <v>520</v>
+      </c>
+      <c r="U49">
+        <v>520</v>
+      </c>
+      <c r="V49">
+        <v>0</v>
+      </c>
+      <c r="W49">
+        <v>0</v>
+      </c>
+      <c r="X49">
+        <v>0</v>
+      </c>
+      <c r="Y49">
+        <v>520</v>
+      </c>
+      <c r="Z49">
+        <v>0</v>
+      </c>
+      <c r="AA49">
+        <v>0</v>
+      </c>
+      <c r="AB49">
         <v>0</v>
       </c>
     </row>
@@ -2656,10 +4742,10 @@
         <v>1</v>
       </c>
       <c r="G50">
-        <v>0.2194987124874836</v>
+        <v>0.2194981032778619</v>
       </c>
       <c r="H50">
-        <v>0.6273575918105793</v>
+        <v>0.627355850605463</v>
       </c>
       <c r="I50">
         <v>0.3498781482089051</v>
@@ -2677,6 +4763,48 @@
         <v>520</v>
       </c>
       <c r="N50">
+        <v>0</v>
+      </c>
+      <c r="O50">
+        <v>520</v>
+      </c>
+      <c r="P50">
+        <v>520</v>
+      </c>
+      <c r="Q50">
+        <v>0</v>
+      </c>
+      <c r="R50">
+        <v>520</v>
+      </c>
+      <c r="S50">
+        <v>1</v>
+      </c>
+      <c r="T50">
+        <v>520</v>
+      </c>
+      <c r="U50">
+        <v>520</v>
+      </c>
+      <c r="V50">
+        <v>0</v>
+      </c>
+      <c r="W50">
+        <v>0</v>
+      </c>
+      <c r="X50">
+        <v>0</v>
+      </c>
+      <c r="Y50">
+        <v>520</v>
+      </c>
+      <c r="Z50">
+        <v>0</v>
+      </c>
+      <c r="AA50">
+        <v>0</v>
+      </c>
+      <c r="AB50">
         <v>0</v>
       </c>
     </row>
@@ -2702,13 +4830,13 @@
         <v>1</v>
       </c>
       <c r="G51">
-        <v>0.1839691741417084</v>
+        <v>0.1839686743308448</v>
       </c>
       <c r="H51">
-        <v>0.5766639688605881</v>
+        <v>0.5766624021692247</v>
       </c>
       <c r="I51">
-        <v>0.3190231817417121</v>
+        <v>0.319023181741712</v>
       </c>
       <c r="J51">
         <v>0.2535699444090383</v>
@@ -2723,6 +4851,48 @@
         <v>520</v>
       </c>
       <c r="N51">
+        <v>0</v>
+      </c>
+      <c r="O51">
+        <v>520</v>
+      </c>
+      <c r="P51">
+        <v>520</v>
+      </c>
+      <c r="Q51">
+        <v>0</v>
+      </c>
+      <c r="R51">
+        <v>520</v>
+      </c>
+      <c r="S51">
+        <v>1</v>
+      </c>
+      <c r="T51">
+        <v>520</v>
+      </c>
+      <c r="U51">
+        <v>520</v>
+      </c>
+      <c r="V51">
+        <v>0</v>
+      </c>
+      <c r="W51">
+        <v>0</v>
+      </c>
+      <c r="X51">
+        <v>0</v>
+      </c>
+      <c r="Y51">
+        <v>520</v>
+      </c>
+      <c r="Z51">
+        <v>0</v>
+      </c>
+      <c r="AA51">
+        <v>0</v>
+      </c>
+      <c r="AB51">
         <v>0</v>
       </c>
     </row>
@@ -2748,10 +4918,10 @@
         <v>1</v>
       </c>
       <c r="G52">
-        <v>0.1794755111202808</v>
+        <v>0.1794750237467796</v>
       </c>
       <c r="H52">
-        <v>0.5783556678103619</v>
+        <v>0.5783540972605692</v>
       </c>
       <c r="I52">
         <v>0.3103203117205888</v>
@@ -2769,6 +4939,48 @@
         <v>520</v>
       </c>
       <c r="N52">
+        <v>0</v>
+      </c>
+      <c r="O52">
+        <v>520</v>
+      </c>
+      <c r="P52">
+        <v>520</v>
+      </c>
+      <c r="Q52">
+        <v>0</v>
+      </c>
+      <c r="R52">
+        <v>520</v>
+      </c>
+      <c r="S52">
+        <v>1</v>
+      </c>
+      <c r="T52">
+        <v>520</v>
+      </c>
+      <c r="U52">
+        <v>520</v>
+      </c>
+      <c r="V52">
+        <v>0</v>
+      </c>
+      <c r="W52">
+        <v>0</v>
+      </c>
+      <c r="X52">
+        <v>0</v>
+      </c>
+      <c r="Y52">
+        <v>520</v>
+      </c>
+      <c r="Z52">
+        <v>0</v>
+      </c>
+      <c r="AA52">
+        <v>0</v>
+      </c>
+      <c r="AB52">
         <v>0</v>
       </c>
     </row>

</xml_diff>